<commit_message>
[auto-snapshot] 2026-04-15 04:00 | onda-hompage | 47 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/동구_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/동구_네일샵.xlsx
@@ -646,7 +646,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="Q17" t="n">
         <v>3</v>
       </c>
       <c r="R17" t="n">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3168,7 +3168,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>yeji4438@naver.com</t>
+          <t>a_nail@naver.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4468,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4750,7 +4750,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4844,7 +4844,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5353,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5592,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5686,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5780,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6058,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6242,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6336,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6653,7 +6653,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6777,13 +6777,13 @@
         </is>
       </c>
       <c r="P68" t="n">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="Q68" t="n">
         <v>1219</v>
       </c>
       <c r="R68" t="n">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="S68" t="inlineStr">
         <is>
@@ -6802,7 +6802,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6896,7 +6896,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -6986,7 +6986,7 @@
       </c>
       <c r="V70" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -7080,7 +7080,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -7268,7 +7268,7 @@
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -7362,7 +7362,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7456,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -7525,13 +7525,13 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q76" t="n">
         <v>3</v>
       </c>
       <c r="R76" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S76" t="inlineStr">
         <is>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-25 16:00 | onda-hompage | 30 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/동구_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/동구_네일샵.xlsx
@@ -432,7 +432,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -646,7 +646,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>jsm90300@naver.com</t>
+          <t>auflaufl@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -888,14 +888,10 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4pjws</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>X</t>
@@ -932,7 +928,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1018,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1112,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1146,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/nail___spring</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1160,7 +1156,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1185,13 +1181,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="Q8" t="n">
         <v>10</v>
       </c>
       <c r="R8" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1210,7 +1206,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1225,11 +1221,7 @@
           <t>뷰티더한_네일</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>fom05@naver.com</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
@@ -1244,7 +1236,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/nail_adorable_heyrin?igsh=c3dqcThsM3Uzb3Uz</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1254,7 +1246,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1264,14 +1256,10 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w5ujgg</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>X</t>
@@ -1308,7 +1296,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1390,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1424,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/queennail1117</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1446,7 +1434,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1496,7 +1484,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1511,11 +1499,7 @@
           <t>the네일샵</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>raphaell1004@naver.com</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
@@ -1590,7 +1574,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1608,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/_naileye__judi?igsh=NnJic3Y2bnl0enVj&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1634,7 +1618,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1644,14 +1628,10 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4sdev</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>X</t>
@@ -1688,7 +1668,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1722,17 +1702,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://pf.kakao.com/_xnIYDxj</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1742,14 +1722,10 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w46f8b</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>O</t>
@@ -1786,7 +1762,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1801,11 +1777,7 @@
           <t>네일 날씨 : 맑음.</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>malgeum_nail@naver.com</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
@@ -1820,17 +1792,17 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://pf.kakao.com/_xhpxedn</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1880,7 +1852,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1946,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -1989,11 +1961,7 @@
           <t>구이일이샵</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>uomdf77@naver.com</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
@@ -2008,7 +1976,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://instagram.com/9212_nail</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2018,7 +1986,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2068,7 +2036,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2070,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/iiidydwn</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2112,24 +2080,20 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wc039a</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>X</t>
@@ -2166,7 +2130,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2181,11 +2145,7 @@
           <t>슈링네일</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>tjddk6025@naver.com</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
@@ -2220,14 +2180,10 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4vjxb</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>X</t>
@@ -2264,7 +2220,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2318,14 +2274,10 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w43muq</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>X</t>
@@ -2362,7 +2314,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2408,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2502,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2584,17 +2536,17 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://pf.kakao.com/_Ukxhxmn</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2604,14 +2556,10 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wm70qab</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>O</t>
@@ -2648,7 +2596,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2682,17 +2630,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://pf.kakao.com/_xhUIxmC</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2702,14 +2650,10 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w5v1lk</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>O</t>
@@ -2746,7 +2690,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2780,17 +2724,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://pf.kakao.com/_HHusxj</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2840,7 +2784,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2814,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/song_rim_dong_nail</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2880,7 +2824,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2930,7 +2874,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2891,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>a_nail@naver.com</t>
+          <t>yeji4438@naver.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -3020,7 +2964,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3035,11 +2979,7 @@
           <t>미다움네일</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>luna_pic@naver.com</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
@@ -3054,7 +2994,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://instagram.com/me_daoom</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3064,7 +3004,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -3114,7 +3054,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3088,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/allroundernail</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3158,24 +3098,20 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w5iwa5</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>X</t>
@@ -3212,7 +3148,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3242,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3276,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/nail.change</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3350,7 +3286,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3360,14 +3296,10 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4d3wc</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>X</t>
@@ -3404,7 +3336,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3370,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://www.instagram.com/banhari0311</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3448,7 +3380,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3458,14 +3390,10 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4x9eu</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>X</t>
@@ -3502,7 +3430,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3524,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3611,11 +3539,7 @@
           <t>이루아네일</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>nec1153@naver.com</t>
-        </is>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
@@ -3668,10 +3592,10 @@
         <v>136</v>
       </c>
       <c r="Q34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R34" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -3690,7 +3614,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3708,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3777,13 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q36" t="n">
         <v>16</v>
       </c>
       <c r="R36" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
@@ -3878,7 +3802,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3892,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4062,7 +3986,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4077,11 +4001,7 @@
           <t>네일맑음</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>s1514@naver.com</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
@@ -4156,7 +4076,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4166,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4260,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4355,11 +4275,7 @@
           <t>고운손</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ghghrjftm@naver.com</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -4405,13 +4321,13 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Q42" t="n">
         <v>2</v>
       </c>
       <c r="R42" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
@@ -4430,7 +4346,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4440,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4534,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4624,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4718,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4817,11 +4733,7 @@
           <t>미추홀구 레벨업 네일뷰티 도화점</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>seeat_f@naver.com</t>
-        </is>
-      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
@@ -4896,7 +4808,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4986,7 +4898,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5080,7 +4992,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5095,11 +5007,7 @@
           <t>라보떼 뷰티</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>dlatmfrl5824@naver.com</t>
-        </is>
-      </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
@@ -5174,7 +5082,7 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5176,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5362,7 +5270,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5377,11 +5285,7 @@
           <t>도화네일</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>gsqnls2u@naver.com</t>
-        </is>
-      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
@@ -5456,7 +5360,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5454,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5619,13 +5523,13 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q55" t="n">
         <v>3</v>
       </c>
       <c r="R55" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="S55" t="inlineStr">
         <is>
@@ -5644,7 +5548,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5738,7 +5642,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5736,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5830,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6020,7 +5924,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6018,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6208,7 +6112,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6151,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -6257,7 +6161,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -6302,7 +6206,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6319,7 +6223,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>nail4season@naver.com</t>
+          <t>gkdisgmlwo@naver.com</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -6371,13 +6275,13 @@
         </is>
       </c>
       <c r="P63" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q63" t="n">
         <v>6</v>
       </c>
       <c r="R63" t="n">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -6396,7 +6300,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6411,11 +6315,7 @@
           <t>로이네일</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>wlgus1647@naver.com</t>
-        </is>
-      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
@@ -6490,7 +6390,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6484,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6599,11 +6499,7 @@
           <t>리마인드뷰티</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>bacsubac@naver.com</t>
-        </is>
-      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
@@ -6678,7 +6574,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6668,7 @@
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6862,7 +6758,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -6877,11 +6773,7 @@
           <t>루미네일 Lumi nail</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>peanutshome02@naver.com</t>
-        </is>
-      </c>
+      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
@@ -6956,7 +6848,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7021,13 +6913,13 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q70" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="R70" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="S70" t="inlineStr">
         <is>
@@ -7046,7 +6938,7 @@
       </c>
       <c r="V70" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7061,11 +6953,7 @@
           <t>바비네일</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>zasd43@naver.com</t>
-        </is>
-      </c>
+      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
@@ -7140,7 +7028,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7230,7 +7118,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7324,7 +7212,7 @@
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7306,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7512,7 +7400,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -7606,7 +7494,7 @@
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>

</xml_diff>